<commit_message>
Add the view hsitory button and also in that popup the next popup of view details of that history searches
</commit_message>
<xml_diff>
--- a/data/Orders_Database.xlsx
+++ b/data/Orders_Database.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -643,6 +643,114 @@
       <c r="L4" t="inlineStr">
         <is>
           <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ORD-1002</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-08-14 20:14:11</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>fjdka</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>lkjlk</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>jkllkj</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ABT-014</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Apple Hair Color (Sachet)</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>100</v>
+      </c>
+      <c r="I5" t="n">
+        <v>300</v>
+      </c>
+      <c r="J5" t="n">
+        <v>30000</v>
+      </c>
+      <c r="K5" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ORD-1003</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-08-14 20:15:14</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>sdfjk</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>kljlkj</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>kljkljlkj</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ABT-015</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Peach Bleach Cream</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>16</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J6" t="n">
+        <v>48000</v>
+      </c>
+      <c r="K6" t="n">
+        <v>48000</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>

</xml_diff>